<commit_message>
added const script and constraints file
</commit_message>
<xml_diff>
--- a/addresses/base_addresses.xlsx
+++ b/addresses/base_addresses.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ME\Desktop\לימודימים\שנה ד\סמס א\‏פרויקט גמר\טבלאות ונתונים\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\routecraft\addresses\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -14,7 +14,7 @@
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>